<commit_message>
Correct jurisdiction label from 'FRANCE' to 'France' (#137) 439d87932185ad57e96ac2e27a751aa18af68cd7
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-mesures-bundle-flux-alimentation-biologie.xlsx
+++ b/main/ig/StructureDefinition-mesures-bundle-flux-alimentation-biologie.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-18T12:52:41+00:00</t>
+    <t>2026-02-23T17:17:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -75,7 +75,7 @@
     <t>Jurisdiction</t>
   </si>
   <si>
-    <t>FRANCE</t>
+    <t>France</t>
   </si>
   <si>
     <t>Description</t>

</xml_diff>

<commit_message>
Update jurisdiction label in sushi-config.yaml 8337f62a5cde8d61ff9b1e87cf5ec9991b21ceb1
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-mesures-bundle-flux-alimentation-biologie.xlsx
+++ b/main/ig/StructureDefinition-mesures-bundle-flux-alimentation-biologie.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-31T09:00:47+00:00</t>
+    <t>2026-05-06T11:42:59+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -75,7 +75,7 @@
     <t>Jurisdiction</t>
   </si>
   <si>
-    <t>France</t>
+    <t>France (la)</t>
   </si>
   <si>
     <t>Description</t>

</xml_diff>